<commit_message>
Docs: D15 -- reconcile Stefaniak citation to 2025 edition across card + tracker
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/ARCH_Method_Reading_Map_Tracker.xlsx
+++ b/Docs/ARCH_Method_Reading_Map_Tracker.xlsx
@@ -588,7 +588,7 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>Stefaniak, J. (n.d.). Using task analysis to inform instructional design. In Design for Learning: Principles, Processes, and Praxis. EdTech Books.
+          <t>Stefaniak, J. E. (2025). Using task analysis to inform instructional design. In J. K. McDonald &amp; R. E. West (Eds.), Design for learning: Principles, processes, and praxis (2025 updated ed.). EdTech Books.
 https://edtechbooks.org/id/task_and_content_analysis</t>
         </is>
       </c>
@@ -861,7 +861,7 @@
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>Stefaniak, J. (n.d.). Using task analysis to inform instructional design. In J. K. McDonald &amp; R. E. West (Eds.), Design for learning: Principles, processes, and praxis. EdTech Books.</t>
+          <t>Stefaniak, J. E. (2025). Using task analysis to inform instructional design. In J. K. McDonald &amp; R. E. West (Eds.), Design for learning: Principles, processes, and praxis (2025 updated ed.). EdTech Books.</t>
         </is>
       </c>
       <c r="C3" s="8" t="inlineStr">

</xml_diff>